<commit_message>
FIX missing BOM entry
</commit_message>
<xml_diff>
--- a/assets/docs/SimpleFOCShieldV1.3/BOM.xlsx
+++ b/assets/docs/SimpleFOCShieldV1.3/BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gospar\Documents\Altium\ArduinoFOC\Project Outputs for ArduinoFOC\Fusion order 2504\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gospar\Documents\NetBeansProjects\antunskuric\assets\docs\SimpleFOCShieldV1.3\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
   <si>
     <t>Designator</t>
   </si>
@@ -135,6 +135,12 @@
   </si>
   <si>
     <t>PULL_A, PULL_B, PULL_I</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>ESR25JZPJ472</t>
   </si>
 </sst>
 </file>
@@ -499,10 +505,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="29.7109375" customWidth="1"/>
     <col min="2" max="2" width="29.85546875" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
     <col min="4" max="4" width="19.5703125" customWidth="1"/>
@@ -695,10 +701,10 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>29</v>
+        <v>37</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="C14" s="3">
         <v>1</v>
@@ -709,10 +715,10 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="C15" s="3">
         <v>1</v>
@@ -723,15 +729,29 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="3">
+        <v>1</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B17" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="3">
-        <v>1</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="C17" s="3">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>34</v>
       </c>
     </row>
@@ -743,15 +763,16 @@
     <hyperlink ref="B9" tooltip="Supplier" display="'"/>
     <hyperlink ref="B10" tooltip="Supplier" display="'"/>
     <hyperlink ref="B11" tooltip="Supplier" display="'"/>
-    <hyperlink ref="B13" tooltip="Supplier" display="'"/>
     <hyperlink ref="B14" tooltip="Supplier" display="'"/>
-    <hyperlink ref="B15" r:id="rId3" tooltip="Supplier" display="'490-TB002-500-03BE"/>
-    <hyperlink ref="B16" r:id="rId4" tooltip="Supplier" display="'490-TB002-500-02BE"/>
+    <hyperlink ref="B15" tooltip="Supplier" display="'"/>
+    <hyperlink ref="B16" r:id="rId3" tooltip="Supplier" display="'490-TB002-500-03BE"/>
+    <hyperlink ref="B17" r:id="rId4" tooltip="Supplier" display="'490-TB002-500-02BE"/>
     <hyperlink ref="B5" tooltip="Supplier" display="'"/>
     <hyperlink ref="B2" tooltip="Supplier" display="'"/>
     <hyperlink ref="B3" tooltip="Supplier" display="'"/>
     <hyperlink ref="B4" tooltip="Supplier" display="'"/>
     <hyperlink ref="B12" tooltip="Supplier" display="'"/>
+    <hyperlink ref="B13" tooltip="Supplier" display="'"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>

</xml_diff>